<commit_message>
cambios de presupuesto, tope por cedula
</commit_message>
<xml_diff>
--- a/docs/exports/Formato_Ejecucion_Pruebas_Portal_Proveedores.xlsx
+++ b/docs/exports/Formato_Ejecucion_Pruebas_Portal_Proveedores.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4466" uniqueCount="2103">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4472" uniqueCount="2109">
   <si>
     <t>Seccion</t>
   </si>
@@ -6336,6 +6336,24 @@
   </si>
   <si>
     <t>Redondear dias en tag de Detalle RFQ</t>
+  </si>
+  <si>
+    <t>Se rompe flujo al cancelar el rfq</t>
+  </si>
+  <si>
+    <t>Solo requisitor deberia ver sus reqs</t>
+  </si>
+  <si>
+    <t>Al crear usuario poner roles en espanol</t>
+  </si>
+  <si>
+    <t>Agregar buscador a los select</t>
+  </si>
+  <si>
+    <t>Se agrego Modal de Ver requisicion para compras</t>
+  </si>
+  <si>
+    <t>Cambiar categoria por subcategoria y ponerla hasta arriba</t>
   </si>
 </sst>
 </file>
@@ -6387,7 +6405,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -6402,6 +6420,12 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -6451,6 +6475,120 @@
         <a:xfrm>
           <a:off x="4229100" y="304800"/>
           <a:ext cx="1476581" cy="771633"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>54925</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>942974</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>409575</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>14858</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Imagen 2"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="4236400" y="1533524"/>
+          <a:ext cx="2793050" cy="1434084"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>4171950</xdr:colOff>
+      <xdr:row>6</xdr:row>
+      <xdr:rowOff>28575</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>352922</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>82</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="4" name="Imagen 3"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="4171950" y="3552825"/>
+          <a:ext cx="3562847" cy="590632"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>9692</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>19050</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>581657</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>20188</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="5" name="Imagen 4"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId4"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="4191167" y="4162425"/>
+          <a:ext cx="3772365" cy="2801488"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -21869,21 +22007,51 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:A2"/>
+  <dimension ref="A1:A8"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="62.7109375" customWidth="1"/>
     <col min="2" max="2" width="25.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
+    <row r="1" spans="1:1" ht="46.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="7" t="s">
         <v>2100</v>
       </c>
     </row>
     <row r="2" spans="1:1" ht="75.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
+      <c r="A2" s="6" t="s">
         <v>2102</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" s="5" customFormat="1" ht="110.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="7" t="s">
+        <v>2107</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A4" s="6" t="s">
+        <v>2103</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A5" s="6" t="s">
+        <v>2104</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A6" s="6" t="s">
+        <v>2105</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1" ht="48.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="6" t="s">
+        <v>2106</v>
+      </c>
+    </row>
+    <row r="8" spans="1:1" ht="220.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="6" t="s">
+        <v>2108</v>
       </c>
     </row>
   </sheetData>

</xml_diff>